<commit_message>
Sefer raporu bildirim denetimi: bildirim baslangictan sonraysa satir sari + Turkce aciklama (21. sutun)
</commit_message>
<xml_diff>
--- a/bos_sablon.xlsx
+++ b/bos_sablon.xlsx
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T5"/>
+  <dimension ref="A1:U5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6.42578125" customWidth="1" style="35" min="1" max="1"/>
@@ -775,6 +775,7 @@
     <col hidden="1" width="15.7109375" customWidth="1" style="35" min="18" max="18"/>
     <col width="21.7109375" bestFit="1" customWidth="1" style="35" min="19" max="19"/>
     <col width="18" customWidth="1" style="35" min="20" max="20"/>
+    <col width="40" customWidth="1" style="35" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -996,6 +997,11 @@
       <c r="T5" s="3" t="inlineStr">
         <is>
           <t>SRC5_Belgeli_Şoför</t>
+        </is>
+      </c>
+      <c r="U5" s="3" t="inlineStr">
+        <is>
+          <t>Bildirim Denetimi</t>
         </is>
       </c>
     </row>

</xml_diff>